<commit_message>
working , need some alteration
</commit_message>
<xml_diff>
--- a/exports/combined_export.xlsx
+++ b/exports/combined_export.xlsx
@@ -417,19 +417,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,11 +486,26 @@
           <t>total_amount</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>credit_note_number</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1_BAHRI-BOLLORE-JED301286.png</t>
+          <t>1_BAHRA-CABLES-60129398.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -497,22 +515,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JED301286</t>
+          <t>60129398</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>02/08/2018</t>
+          <t>02.01.2019</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bahri Bollore Logistics</t>
+          <t>Bahra Advanced Cable Manufacture Co Lid</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
+          <t>The Civil Works Joint Venture Of Saudi Arabian Bechtel Company</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -520,20 +538,17 @@
           <t>SAR</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>7589.75</v>
-      </c>
-      <c r="I2" t="n">
-        <v>210</v>
-      </c>
-      <c r="J2" t="n">
-        <v>7799.75</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20220820_160841493.jpg</t>
+          <t>1_BAHRI-BOLLORE-JED301286.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -543,33 +558,77 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>310426975200003</t>
+          <t>TAX INVOICE JED301286</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>21/07/2022</t>
+          <t>02/08/2018</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>مطعم طريق المطار</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Bahri Bollore Logistics</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>41.74</v>
+        <v>7799.75</v>
       </c>
       <c r="I3" t="n">
-        <v>6.26</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>48</v>
+        <v>7799.75</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4_JY2020-07-JV000756.png</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>credit_note</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>المشترك للاعمل المدنى</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>01-2422</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>31/03/2020</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1417.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working, needs to be fixed
</commit_message>
<xml_diff>
--- a/exports/combined_export.xlsx
+++ b/exports/combined_export.xlsx
@@ -422,10 +422,10 @@
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="41" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1_BAHRA-CABLES-60129398.png</t>
+          <t>1_BAHRI-BOLLORE-JED301286.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -515,22 +515,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>60129398</t>
+          <t>JED301286</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>02.01.2019</t>
+          <t>02/08/2018</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bahra Advanced Cable Manufacture Co Lid</t>
+          <t>Bahri Bollore Logistics</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The Civil Works Joint Venture Of Saudi Arabian Bechtel Company</t>
+          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -538,9 +538,15 @@
           <t>SAR</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>7589.75</v>
+      </c>
+      <c r="I2" t="n">
+        <v>210</v>
+      </c>
+      <c r="J2" t="n">
+        <v>7799.75</v>
+      </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
@@ -548,88 +554,78 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1_BAHRI-BOLLORE-JED301286.png</t>
+          <t>4_JY2020-07-JV000756.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>invoice</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TAX INVOICE JED301286</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>02/08/2018</t>
-        </is>
-      </c>
+          <t>credit_note</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bahri Bollore Logistics</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>7799.75</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>7799.75</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+          <t>المشترك للاعمل المدنى</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>01-2422</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>31/03/2020</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1417.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4_JY2020-07-JV000756.png</t>
+          <t>20220820_161037175.jpg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>credit_note</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+          <t>invoice</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>T0٠٠٠٠</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>٠٤ ١</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>المشترك للاعمل المدنى</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>AIRPORT SERVICE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mr / Ms</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>01-2422</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>31/03/2020</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>1417.5</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
working, Ready to deploy
</commit_message>
<xml_diff>
--- a/exports/combined_export.xlsx
+++ b/exports/combined_export.xlsx
@@ -417,15 +417,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="69" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
@@ -487,7 +487,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1_BAHRI-BOLLORE-JED301286.png</t>
+          <t>1_CPS-CONSTRUCTION-PLANT-490.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -497,43 +497,41 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JED301286</t>
+          <t>490</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>02/08/2018</t>
+          <t>17.10.2018</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bahri Bollore Logistics</t>
+          <t>CPS CONSTRUCTION PLANT SERVICE GMBH</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
+          <t>Almabani General Contractors</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SAR</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>7589.75</v>
-      </c>
-      <c r="I2" t="n">
-        <v>210</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>7799.75</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20220820_161037175.jpg</t>
+          <t>1_BAHRI-BOLLORE-JED301286.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -543,28 +541,84 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>T0٠٠٠٠</t>
+          <t>JED301286</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>٠٤ ١</t>
+          <t>2018-08-02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AIRPORT SERVICE</t>
+          <t>BAHRI BOLLORE LOGISTICS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Mr / Ms</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+          <t>RIYADH METRO PROJECT CIVIL WORKS JOINT</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>7589.75</v>
+      </c>
+      <c r="I3" t="n">
+        <v>210</v>
+      </c>
+      <c r="J3" t="n">
+        <v>7799.75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4_JY2020-07-JV000738.png</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>invoice</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>200024783</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>29/02/2020</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SODAMCO Industrial Company for Construction Chemicals W.L.L</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>C،W J المشروع المشترك لشركة بكتل العربية والمباني وإتحاد المقاولون</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1501.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>75.075</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1576.575</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>